<commit_message>
Update job sources and profile keywords
</commit_message>
<xml_diff>
--- a/daily_jobs.xlsx
+++ b/daily_jobs.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Intern Data Analyst (New Engines Department)</t>
+          <t>Internship - DAT Industrialization</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Zürich, Switzerland</t>
+          <t>Switzerland, Zürich</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -538,15 +538,15 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/e4253136-b35a-42f9-8c7d-d76be6384e0d</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/c6014db5-c37c-4b5f-b37c-2333b1f58759</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>analyst, business development, intern, switzerland</t>
+          <t>business development, intern, internship, switzerland</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -564,7 +564,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Internship - DAT Industrialization</t>
+          <t>Intern Data Analyst (New Engines Department)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Switzerland, Zürich</t>
+          <t>Zürich, Switzerland</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -584,15 +584,15 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/c6014db5-c37c-4b5f-b37c-2333b1f58759</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/e4253136-b35a-42f9-8c7d-d76be6384e0d</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>business development, intern, internship, switzerland</t>
+          <t>analyst, business development, intern, switzerland</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -652,41 +652,41 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Marketing Cloud Account Executive</t>
+          <t>Founders Associate Marketing &amp; Commercial (m/w/d)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>salesforce.com Sàrl</t>
+          <t>hellomateo</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Switzerland - Zurich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>jobs.ch Business Development Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/76afa31f-e54f-4912-99ff-a6ac9cea24dc</t>
+          <t>https://www.arbeitnow.com/jobs/companies/hellomateo/founders-associate-marketing-commercial-berlin-380297</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>business development, marketing, sales, switzerland, zurich</t>
+          <t>associate, berlin, commercial, germany, marketing</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>role fit; strong keyword match; target location</t>
+          <t>role fit; strong keyword match; target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -698,27 +698,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Growth Marketing Specialist (m(w/d)</t>
+          <t>Marketing Cloud Account Executive</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>VDB Digital GmbH</t>
+          <t>salesforce.com Sàrl</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Osnabrück</t>
+          <t>Switzerland - Zurich</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobs.ch Business Development Switzerland</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vdb-digital-gmbh/growth-marketing-specialist-mw-d-osnabruck-259781</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/76afa31f-e54f-4912-99ff-a6ac9cea24dc</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>germany, growth, growth marketing, marketing</t>
+          <t>business development, marketing, sales, switzerland, zurich</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -744,35 +744,35 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Service Sales Engineer – Transformer Service (Traction/Rail) 80 - 100% (f/m/d)</t>
+          <t>Growth Marketing Specialist (m(w/d)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>VDB Digital GmbH</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Satigny, Geneva, Switzerland</t>
+          <t>Osnabrück</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>jobs.ch Business Development Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/b2dc5b37-5212-4ea3-b563-be2643a61dc1</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vdb-digital-gmbh/growth-marketing-specialist-mw-d-osnabruck-259781</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>business development, geneva, sales, switzerland</t>
+          <t>germany, growth, growth marketing, marketing</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -1020,17 +1020,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Research Scientist in Machine Perception (80 -100%)</t>
+          <t>Service Sales Engineer – Transformer Service (Traction/Rail) 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ABB Schweiz AG</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Baden-Daettwil, Aargau, Switzerland</t>
+          <t>Satigny, Geneva, Switzerland</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1040,15 +1040,15 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/dcd1137e-0d79-4945-a13c-fda36a08b2c3</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/b2dc5b37-5212-4ea3-b563-be2643a61dc1</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>business development, switzerland</t>
+          <t>business development, geneva, sales, switzerland</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1066,17 +1066,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Customer Support Engineer</t>
+          <t>Research Scientist in Machine Perception (80 -100%)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SR Technics Switzerland AG</t>
+          <t>ABB Schweiz AG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Zürich, Switzerland</t>
+          <t>Baden-Daettwil, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/c59db4a2-bb01-45ed-a6b9-a5f94fdbfc06</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/dcd1137e-0d79-4945-a13c-fda36a08b2c3</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Logistics Specialist</t>
+          <t>Customer Support Engineer</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/89ad1c96-37b9-4940-bf0c-9599bcc056fa</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/c59db4a2-bb01-45ed-a6b9-a5f94fdbfc06</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
@@ -1158,17 +1158,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Service Project &amp; Tender Specialist 80 – 100% (f/m/d)</t>
+          <t>Logistics Specialist</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>SR Technics Switzerland AG</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Turgi, Aargau, Switzerland</t>
+          <t>Zürich, Switzerland</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/0a05e76b-0985-4dd3-87f4-3d9175daa2c7</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/89ad1c96-37b9-4940-bf0c-9599bcc056fa</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -1204,17 +1204,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Supervisor Logistics</t>
+          <t>Service Project &amp; Tender Specialist 80 – 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>SR Technics Switzerland AG</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Bad Zurzach, Switzerland</t>
+          <t>Turgi, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/0de73426-551d-472e-a065-57e08455f6ea</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/0a05e76b-0985-4dd3-87f4-3d9175daa2c7</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Process Engineer</t>
+          <t>Supervisor Logistics</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Zürich, Switzerland</t>
+          <t>Bad Zurzach, Switzerland</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/a70a1155-eebb-407c-99a2-2c6ccabbfa22</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/0de73426-551d-472e-a065-57e08455f6ea</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
@@ -1296,41 +1296,41 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Marketing Trainee</t>
+          <t>Process Engineer</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Swibeco AG</t>
+          <t>SR Technics Switzerland AG</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Lausanne, Waadt, Switzerland</t>
+          <t>Zürich, Switzerland</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>jobs.ch Business Development Switzerland</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9d3f6b3d-8e94-4e58-9c54-694f9db91205</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/a70a1155-eebb-407c-99a2-2c6ccabbfa22</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>lausanne, marketing, switzerland, trainee</t>
+          <t>business development, switzerland</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit</t>
+          <t>role fit; strong keyword match; target location</t>
         </is>
       </c>
     </row>
@@ -1342,41 +1342,41 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Online Marketing Trainee</t>
+          <t>Marketing Trainee</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Cyrus Digital GmbH</t>
+          <t>Swibeco AG</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Lausanne, Waadt, Switzerland</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
+          <t>https://www.jobup.ch/en/jobs/detail/9d3f6b3d-8e94-4e58-9c54-694f9db91205</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich, trainee</t>
+          <t>lausanne, marketing, switzerland, trainee</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -1388,17 +1388,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Growth Marketing Manager / Performance Marketing Manager (m/w/d) | 100 % Remote, bis zu 75k &amp; moderner Marketing Stack</t>
+          <t>Online Marketing Trainee</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>RX-WATERTEC GmbH</t>
+          <t>Cyrus Digital GmbH</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Karlsruhe</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1408,25 +1408,21 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/rx-watertec-gmbh/growth-marketing-manager-performance-marketing-manager-100-remote-bis-zu-75k-moderner-marketing-stack-karlsruhe-413521</t>
+          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>germany, growth, growth marketing, marketing, remote</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
-        </is>
-      </c>
+          <t>germany, marketing, munich, trainee</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>role fit; strong keyword match; target location; seniority warning</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -1438,35 +1434,35 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Named Account Manager - Retail &amp; CG (Consumer Goods)</t>
+          <t>Growth Marketing Manager / Performance Marketing Manager (m/w/d) | 100 % Remote, bis zu 75k &amp; moderner Marketing Stack</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>salesforce.com Sàrl</t>
+          <t>RX-WATERTEC GmbH</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Switzerland - Zurich</t>
+          <t>Karlsruhe</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>jobs.ch Business Development Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/bc0d2bb9-5573-4da2-86f8-ce424ad1d623</t>
+          <t>https://www.arbeitnow.com/jobs/companies/rx-watertec-gmbh/growth-marketing-manager-performance-marketing-manager-100-remote-bis-zu-75k-moderner-marketing-stack-karlsruhe-413521</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>business development, sales, switzerland, zurich</t>
+          <t>germany, growth, growth marketing, marketing, remote</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1488,17 +1484,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Territory Sales Manager 80 – 100% (f/m/d)</t>
+          <t>Head of Product - Consumer (Private Customer) (f|m|d) | 100% | Hybrid working model | Zurich Switzerland</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>SMG Swiss Marketplace Group</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1508,7 +1504,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/32b4f7fe-52e3-40b9-a631-59bd1f283719</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/e4afae49-fa88-4b01-adad-2363f5990c87</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
@@ -1516,12 +1512,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>business development, sales, switzerland, zurich</t>
+          <t>business development, product, switzerland, zurich</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>head of</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1538,17 +1534,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Area Sales Manager 80 - 100% (f/m/d)</t>
+          <t>Named Account Manager - Retail &amp; CG (Consumer Goods)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>salesforce.com Sàrl</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Switzerland - Zurich</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1558,7 +1554,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/3ef91e75-64e7-48a3-b2e4-69b9c352c007</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/bc0d2bb9-5573-4da2-86f8-ce424ad1d623</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
@@ -1588,17 +1584,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Business Development Manager Infrastruktur, 100%</t>
+          <t>Territory Sales Manager 80 – 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Saint Gobain Schweiz</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1608,15 +1604,15 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/4a51eb62-3d06-437a-8a70-194c724c4f6d</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/32b4f7fe-52e3-40b9-a631-59bd1f283719</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>business development, switzerland</t>
+          <t>business development, sales, switzerland, zurich</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1638,17 +1634,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Head of Product - Consumer (Private Customer) (f|m|d) | 100% | Hybrid working model | Zurich Switzerland</t>
+          <t>Area Sales Manager 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>SMG Swiss Marketplace Group</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1658,20 +1654,20 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/e4afae49-fa88-4b01-adad-2363f5990c87</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/3ef91e75-64e7-48a3-b2e4-69b9c352c007</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>business development, switzerland, zurich</t>
+          <t>business development, sales, switzerland, zurich</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>head of</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -1688,12 +1684,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Business Development Manager D-CH</t>
+          <t>Business Development Manager Infrastruktur, 100%</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>ELCA Security SA</t>
+          <t>Saint Gobain Schweiz</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1708,7 +1704,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/7611996a-66a2-4e5d-8493-12b5234e8d58</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/4a51eb62-3d06-437a-8a70-194c724c4f6d</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
@@ -1738,17 +1734,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Project Manager - Environmental Remediation / Contaminated Sites</t>
+          <t>Cybersecurity Business Development Manager D-CH</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>ERM Swiss GmbH</t>
+          <t>ELCA Security SA</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Lausanne, Switzerland</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1758,7 +1754,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/ff31274f-59e3-4c1f-b0dd-b69184e4f1d8</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/7611996a-66a2-4e5d-8493-12b5234e8d58</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
@@ -1766,7 +1762,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>business development, lausanne, switzerland</t>
+          <t>business development, switzerland</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1788,17 +1784,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Account Manager - Switzerland</t>
+          <t>Project Manager - Environmental Remediation / Contaminated Sites</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Agilent Technologies (Schweiz) AG</t>
+          <t>ERM Swiss GmbH</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Switzerland-Basel</t>
+          <t>Lausanne, Switzerland</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1808,7 +1804,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/4056f76a-0938-4010-b43b-7f131f2ece00</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/ff31274f-59e3-4c1f-b0dd-b69184e4f1d8</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
@@ -1816,7 +1812,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>basel, business development, switzerland</t>
+          <t>business development, lausanne, switzerland</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -1838,17 +1834,17 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Project Manager Engineering 80 – 100% (f/m/d)</t>
+          <t>Account Manager - Switzerland</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>Agilent Technologies (Schweiz) AG</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Turgi, Aargau, Switzerland</t>
+          <t>Switzerland-Basel</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1858,7 +1854,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/7d776c0c-ebf7-4cad-be67-38b98e8ddd70</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/4056f76a-0938-4010-b43b-7f131f2ece00</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
@@ -1866,7 +1862,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>business development, switzerland</t>
+          <t>basel, business development, switzerland</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1888,41 +1884,45 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>ECS Account Executive</t>
+          <t>Project Manager Engineering 80 – 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>salesforce.com Sàrl</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Switzerland - Zurich</t>
+          <t>Turgi, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>jobs.ch Business Development Switzerland</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9a399eaa-b558-4562-b057-89c29757c221</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/7d776c0c-ebf7-4cad-be67-38b98e8ddd70</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>marketing, sales, switzerland, zurich</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr"/>
+          <t>business development, switzerland</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>role fit; strong keyword match; target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -1934,41 +1934,41 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Data360 &amp; Agentforce Architects</t>
+          <t>WerkstudentIn Marketing</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>salesforce.com Sàrl</t>
+          <t>amc Group</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Switzerland - Zurich</t>
+          <t>Bonn</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/4f41c31f-ee22-425d-8ea5-9469a703e656</t>
+          <t>https://www.arbeitnow.com/jobs/companies/amc-group/werkstudentin-marketing-bonn-489915</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>marketing, sales, switzerland, zurich</t>
+          <t>germany, marketing, werkstudent</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -1980,15 +1980,19 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Data Analyst, Marketing</t>
+          <t>Werkstudent (m/w/d) Recruiting &amp; Marketing</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Quince</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
+          <t>Burner Marketing GmbH</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Erlangen</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Arbeitnow Marketing Germany</t>
@@ -1996,21 +2000,21 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/quince/data-analyst-marketing-450463</t>
+          <t>https://www.arbeitnow.com/jobs/companies/burner-marketing-gmbh/werkstudent-recruiting-marketing-erlangen-142686</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>analyst, germany, marketing</t>
+          <t>germany, marketing, werkstudent</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2026,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Werkstudent Marketing (all genders) für reev</t>
+          <t>Praktikum Online-Marketing (All Gender)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Future Energy Ventures</t>
+          <t>CONTXT Online-Marketing GmbH</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Ober-Ramstadt</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2042,21 +2046,21 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/future-energy-ventures/werkstudent-marketing-all-genders-fur-reev-munich-399557</t>
+          <t>https://www.arbeitnow.com/jobs/companies/contxt-online-marketing-gmbh/praktikum-online-marketing-all-gender-ober-ramstadt-369542</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich, venture</t>
+          <t>germany, marketing, praktikum</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2068,17 +2072,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Marketing Analyst</t>
+          <t>Werkstudent Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Custom Surgical GmbH</t>
+          <t>GSG Berlin GmbH</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2088,21 +2092,21 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/custom-surgical-gmbh/marketing-analyst-munich-145698</t>
+          <t>https://www.arbeitnow.com/jobs/companies/gsg-berlin-gmbh/werkstudent-marketing-berlin-288513</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>analyst, germany, marketing, munich</t>
+          <t>berlin, germany, marketing, werkstudent</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2114,17 +2118,17 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Junior Online Marketing Manager</t>
+          <t>Praktikum Online-Marketing / Marketing / KI / AI</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Cyrus Digital GmbH</t>
+          <t>SEOMATIK GmbH</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Bielefeld</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2134,25 +2138,21 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/junior-online-marketing-manager-munich-311721</t>
+          <t>https://www.arbeitnow.com/jobs/companies/seomatik-gmbh/praktikum-online-marketing-marketing-ki-ai-bielefeld-477843</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>germany, junior, marketing, munich</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
-        </is>
-      </c>
+          <t>germany, marketing, praktikum</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit; seniority warning</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2164,41 +2164,41 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Production Controller 80 - 100% (f/m/d)</t>
+          <t>Pflichtpraktikum (Content-)Marketing [ab 15.09.26]</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>frechekoepfe GmbH</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Karlsruhe</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/7b1a971b-50a1-41da-9b11-e10ae50af267</t>
+          <t>https://www.arbeitnow.com/jobs/companies/frechekoepfe-gmbh/pflichtpraktikum-content-marketing-ab-150926-karlsruhe-243979</t>
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>marketing, switzerland, zurich</t>
+          <t>germany, marketing, praktikum</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2210,17 +2210,17 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Marketing Assistent</t>
+          <t>Werkstudent Marketing (all genders) für reev</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Henning Marketing</t>
+          <t>Future Energy Ventures</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Rosenheim</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2230,21 +2230,21 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/henning-marketing/marketing-assistent-rosenheim-346483</t>
+          <t>https://www.arbeitnow.com/jobs/companies/future-energy-ventures/werkstudent-marketing-all-genders-fur-reev-munich-399557</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>germany, marketing, munich, werkstudent</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2256,17 +2256,17 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Performance Marketing Specialist (m/w/d) | 100% Homeoffice</t>
+          <t>Werkstudent (m/w/d) Social Media Marketing</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Online Marketing United GmbH</t>
+          <t>spized GmbH</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Braunschweig</t>
+          <t>Cologne</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2276,21 +2276,21 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/online-marketing-united-gmbh/performance-marketing-specialist-100-homeoffice-braunschweig-393785</t>
+          <t>https://www.arbeitnow.com/jobs/companies/spized-gmbh/werkstudent-social-media-marketing-cologne-91270</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>germany, marketing, werkstudent</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>WerkstudentIn Marketing</t>
+          <t>Production Controller 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>amc Group</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Bonn</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/amc-group/werkstudentin-marketing-bonn-489915</t>
+          <t>https://www.jobup.ch/en/jobs/detail/7b1a971b-50a1-41da-9b11-e10ae50af267</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
@@ -2330,13 +2330,13 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>marketing, product, switzerland, zurich</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2348,27 +2348,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Werkstudent (m/w/d) Recruiting &amp; Marketing</t>
+          <t>ECS Account Executive</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Burner Marketing GmbH</t>
+          <t>salesforce.com Sàrl</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Erlangen</t>
+          <t>Switzerland - Zurich</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/burner-marketing-gmbh/werkstudent-recruiting-marketing-erlangen-142686</t>
+          <t>https://www.jobup.ch/en/jobs/detail/9a399eaa-b558-4562-b057-89c29757c221</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
@@ -2376,13 +2376,13 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>marketing, sales, switzerland, zurich</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2394,27 +2394,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Assistenz (m/w/d) Online-Marketing</t>
+          <t>Data360 &amp; Agentforce Architects</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Marketing Juwel GmbH</t>
+          <t>salesforce.com Sàrl</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Switzerland - Zurich</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/marketing-juwel-gmbh/assistenz-online-marketing-berlin-327213</t>
+          <t>https://www.jobup.ch/en/jobs/detail/4f41c31f-ee22-425d-8ea5-9469a703e656</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
@@ -2422,13 +2422,13 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>marketing, sales, switzerland, zurich</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2440,27 +2440,23 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Online-Marketing (All Gender)</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>CONTXT Online-Marketing GmbH</t>
-        </is>
-      </c>
+          <t>Audience and partnerships editor</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Ober-Ramstadt</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/contxt-online-marketing-gmbh/praktikum-online-marketing-all-gender-ober-ramstadt-369542</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/editing-translation-positions/audience-and-partnerships-editor/tp8Ey5roXuZNKu4CCTC2NG</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
@@ -2468,7 +2464,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>amsterdam, netherlands, partnerships</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2486,19 +2482,15 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Werkstudent Marketing (m/w/d)</t>
+          <t>Data Analyst, Marketing</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>GSG Berlin GmbH</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Berlin</t>
-        </is>
-      </c>
+          <t>Quince</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Arbeitnow Marketing Germany</t>
@@ -2506,7 +2498,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/gsg-berlin-gmbh/werkstudent-marketing-berlin-288513</t>
+          <t>https://www.arbeitnow.com/jobs/companies/quince/data-analyst-marketing-450463</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
@@ -2514,13 +2506,13 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>analyst, germany, marketing</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2532,17 +2524,17 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Online-Marketing / Marketing / KI / AI</t>
+          <t>Marketing Analyst</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>SEOMATIK GmbH</t>
+          <t>Custom Surgical GmbH</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Bielefeld</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2552,7 +2544,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/seomatik-gmbh/praktikum-online-marketing-marketing-ki-ai-bielefeld-477843</t>
+          <t>https://www.arbeitnow.com/jobs/companies/custom-surgical-gmbh/marketing-analyst-munich-145698</t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
@@ -2560,13 +2552,13 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>analyst, germany, marketing, munich</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2578,41 +2570,45 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Pflichtpraktikum (Content-)Marketing [ab 15.09.26]</t>
+          <t>Lead Health Systems Integrations Manager, International</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>frechekoepfe GmbH</t>
+          <t>Exact Sciences International Sàrl</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Karlsruhe</t>
+          <t>Switzerland - Zug</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/frechekoepfe-gmbh/pflichtpraktikum-content-marketing-ab-150926-karlsruhe-243979</t>
+          <t>https://www.jobup.ch/en/jobs/detail/ee1716cf-4f51-484a-9948-f5498c9bd8c3</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr"/>
+          <t>intern, international, marketing, switzerland, zug</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>lead, manager</t>
+        </is>
+      </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>strong keyword match; target location; junior/internship fit; seniority warning</t>
         </is>
       </c>
     </row>
@@ -2624,41 +2620,37 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Werkstudent (m/w/d) Social Media Marketing</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>spized GmbH</t>
-        </is>
-      </c>
+          <t>Sales Coordinator | German or Dutch | Noord-Holland</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Cologne</t>
+          <t>Enkhuizen</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/spized-gmbh/werkstudent-social-media-marketing-cologne-91270</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/sales-positions/sales-coordinator-german-or-dutch-noord-holland/qwMFTL8BTcNJMMrM7YzcHQ</t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>netherlands, sales</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2670,41 +2662,37 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Praktikant im Digital Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>MSC Cruises GmbH</t>
-        </is>
-      </c>
+          <t>Inside Sales Representative – French &amp; English</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Mijdrecht</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/msc-cruises-gmbh/praktikant-im-digital-marketing-munich-101650</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/customer-service-positions/inside-sales-representative-–-french-english/6ScLxSBfWnjvq3qcNRFzwp</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich</t>
+          <t>netherlands, sales</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2716,17 +2704,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>(Pflicht-) Praktikant Marketing (w/m/d) (100%)</t>
+          <t>Marketing Assistent</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>HighCoordination GmbH</t>
+          <t>Henning Marketing</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Singen</t>
+          <t>Rosenheim</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2736,11 +2724,11 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/highcoordination-gmbh/pflicht-praktikant-marketing-100-singen-161583</t>
+          <t>https://www.arbeitnow.com/jobs/companies/henning-marketing/marketing-assistent-rosenheim-346483</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2750,7 +2738,7 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2762,37 +2750,41 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Audience and partnerships editor</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr"/>
+          <t>Performance Marketing Specialist (m/w/d) | 100% Homeoffice</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Online Marketing United GmbH</t>
+        </is>
+      </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Braunschweig</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/editing-translation-positions/audience-and-partnerships-editor/tp8Ey5roXuZNKu4CCTC2NG</t>
+          <t>https://www.arbeitnow.com/jobs/companies/online-marketing-united-gmbh/performance-marketing-specialist-100-homeoffice-braunschweig-393785</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>amsterdam, netherlands, partnerships</t>
+          <t>germany, marketing</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2804,23 +2796,27 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Sales Coordinator | German or Dutch | Noord-Holland</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr"/>
+          <t>Assistenz (m/w/d) Online-Marketing</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Juwel GmbH</t>
+        </is>
+      </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Enkhuizen</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/sales-positions/sales-coordinator-german-or-dutch-noord-holland/qwMFTL8BTcNJMMrM7YzcHQ</t>
+          <t>https://www.arbeitnow.com/jobs/companies/marketing-juwel-gmbh/assistenz-online-marketing-berlin-327213</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
@@ -2828,7 +2824,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>netherlands, sales</t>
+          <t>berlin, germany, marketing</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -2846,23 +2842,27 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Inside Sales Representative – French &amp; English</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr"/>
+          <t>Praktikant im Digital Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>MSC Cruises GmbH</t>
+        </is>
+      </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Mijdrecht</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/customer-service-positions/inside-sales-representative-–-french-english/6ScLxSBfWnjvq3qcNRFzwp</t>
+          <t>https://www.arbeitnow.com/jobs/companies/msc-cruises-gmbh/praktikant-im-digital-marketing-munich-101650</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>netherlands, sales</t>
+          <t>germany, marketing, munich</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -2888,45 +2888,41 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Lead Health Systems Integrations Manager, International</t>
+          <t>(Pflicht-) Praktikant Marketing (w/m/d) (100%)</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Exact Sciences International Sàrl</t>
+          <t>HighCoordination GmbH</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Switzerland - Zug</t>
+          <t>Singen</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/ee1716cf-4f51-484a-9948-f5498c9bd8c3</t>
+          <t>https://www.arbeitnow.com/jobs/companies/highcoordination-gmbh/pflicht-praktikant-marketing-100-singen-161583</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>intern, marketing, switzerland</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>lead, manager</t>
-        </is>
-      </c>
+          <t>germany, marketing</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit; seniority warning</t>
+          <t>target location</t>
         </is>
       </c>
     </row>
@@ -2938,37 +2934,45 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Assistant Financial Controller | English | Almere area</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr"/>
+          <t>Junior Online Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Cyrus Digital GmbH</t>
+        </is>
+      </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Almere</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/finance-accounting-positions/assistant-financial-controller-english-almere-area/io2zwMAJH8NAJsCQGtpojm</t>
+          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/junior-online-marketing-manager-munich-311721</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr"/>
+          <t>germany, junior, marketing, munich</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>target location</t>
+          <t>target location; junior/internship fit; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3008,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
+          <t>netherlands, rotterdam</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3232,7 +3236,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Java Backend Engineer (Kotlin) - Freelance/zzp</t>
+          <t>Test Automation Engineer - freelance/zzp</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
@@ -3248,7 +3252,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/java-backend-engineer-kotlin-freelancezzp/kP1rMZUuK5tXV3FkBKWGuV</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/test-automation-engineer-freelancezzp/qHDAgcfjd9oSGj8gLMFqV6</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
@@ -3274,13 +3278,13 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Test Automation Engineer - freelance/zzp</t>
+          <t>Logistics &amp; Returns Coordinator | French C2</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Breda</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3290,7 +3294,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/test-automation-engineer-freelancezzp/qHDAgcfjd9oSGj8gLMFqV6</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/supply-chain-logistics-positions/logistics-returns-coordinator-french-c2/8jZ9pvyDfbqCVoy5r7V8F7</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
@@ -3298,7 +3302,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>amsterdam, netherlands</t>
+          <t>netherlands</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3316,13 +3320,13 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Java Backend Engineer (Kotlin) - Temporary</t>
+          <t>Customer Service Representative | German C2</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Eindhoven</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3332,7 +3336,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/java-backend-engineer-kotlin-temporary/oQs6kAvwDoSinBavtghURc</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/customer-service-positions/customer-service-representative-german-c2/wZ5cX8YbBsjkBwC1Q3LEj4</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
@@ -3340,7 +3344,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>amsterdam, netherlands</t>
+          <t>eindhoven, netherlands</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3358,13 +3362,13 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Logistics &amp; Returns Coordinator | French C2</t>
+          <t>Platform Security Engineer</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Breda</t>
+          <t>Rotterdam Permanent</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3374,7 +3378,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/supply-chain-logistics-positions/logistics-returns-coordinator-french-c2/8jZ9pvyDfbqCVoy5r7V8F7</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/platform-security-engineer/owpdvmCHTRCBcCLu211kAc</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
@@ -3382,7 +3386,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
+          <t>netherlands, rotterdam</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3400,13 +3404,13 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Customer Service Representative | German C2</t>
+          <t>Electrical Technician – 5-Star Hotel</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Eindhoven</t>
+          <t>Amsterdam Permanent</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3416,7 +3420,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/customer-service-positions/customer-service-representative-german-c2/wZ5cX8YbBsjkBwC1Q3LEj4</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/other-positions/electrical-technician-–-5-star-hotel/bx82JreNcUNcomkxzzk4Jb</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
@@ -3424,7 +3428,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
+          <t>amsterdam, netherlands</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
@@ -3442,37 +3446,45 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Platform Security Engineer</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr"/>
+          <t>Marketing Operations Manager (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>bits&amp;birds GmbH</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Rotterdam Permanent</t>
+          <t>Künzell</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/platform-security-engineer/owpdvmCHTRCBcCLu211kAc</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bitsbirds-gmbh/marketing-operations-manager-kunzell-83103</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr"/>
+          <t>germany, marketing, operations</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>target location</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3484,37 +3496,45 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>DevOps Engineer - SIP Core (Voice Platform)</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr"/>
+          <t>Improvement Project Manager – Data &amp; Digital Analytics 80 – 100% (f/m/d)</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Hitachi Energy AG</t>
+        </is>
+      </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Rotterdam Temporary</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/devops-engineer-sip-core-voice-platform/sGfXBGvCBQ2Vdqa6CTH62X</t>
+          <t>https://www.jobup.ch/en/jobs/detail/e519db1d-4d90-4cd9-86ef-207e574bd548</t>
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr"/>
+          <t>marketing, switzerland, zurich</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>manager</t>
+        </is>
+      </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
-          <t>target location</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3526,37 +3546,45 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Electrical Technician – 5-Star Hotel</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr"/>
+          <t>Senior Trademark Counsel</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Abbott AG</t>
+        </is>
+      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Amsterdam Permanent</t>
+          <t>Switzerland &amp;gt; Allschwil : H-127</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/other-positions/electrical-technician-–-5-star-hotel/bx82JreNcUNcomkxzzk4Jb</t>
+          <t>https://www.jobup.ch/en/jobs/detail/53ab1fe0-9943-4f79-b255-922cd5756dd8</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>amsterdam, netherlands</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr"/>
+          <t>marketing, switzerland</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>senior</t>
+        </is>
+      </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>target location</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3568,35 +3596,35 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Marketing Operations Manager (m/w/d)</t>
+          <t>Category Manager Apple/Mobile (m/w/d)</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>bits&amp;birds GmbH</t>
+          <t>TD SYNNEX Switzerland GmbH</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Künzell</t>
+          <t>Rotkreuz, Switzerland</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>jobup.ch Marketing Switzerland</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bitsbirds-gmbh/marketing-operations-manager-kunzell-83103</t>
+          <t>https://www.jobup.ch/en/jobs/detail/83432ecd-3dd3-4a98-9663-6f678ad52a5e</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, operations</t>
+          <t>marketing, switzerland</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3606,7 +3634,7 @@
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3618,17 +3646,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Improvement Project Manager – Data &amp; Digital Analytics 80 – 100% (f/m/d)</t>
+          <t>Global Medical Director Cardiometabolic</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>Abbott AG</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Switzerland &amp;gt; Allschwil : H-127</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3638,25 +3666,25 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/e519db1d-4d90-4cd9-86ef-207e574bd548</t>
+          <t>https://www.jobup.ch/en/jobs/detail/9e624f50-f1d8-4017-b805-17a8f78d7acd</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>marketing, switzerland, zurich</t>
+          <t>marketing, switzerland</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>director</t>
         </is>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3668,17 +3696,17 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Senior Trademark Counsel</t>
+          <t>Finance and Administration Manager</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Abbott AG</t>
+          <t>Fairmont Grand Hôtel Geneva</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Switzerland &amp;gt; Allschwil : H-127</t>
+          <t>Hotel Rotary Geneva - MGallery, Geneva, Switzerland</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -3688,25 +3716,25 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/53ab1fe0-9943-4f79-b255-922cd5756dd8</t>
+          <t>https://www.jobup.ch/en/jobs/detail/0996602f-337e-48a0-a447-50bc3dbec7b2</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>marketing, switzerland</t>
+          <t>geneva, marketing, switzerland</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3718,17 +3746,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Category Manager Apple/Mobile (m/w/d)</t>
+          <t>R&amp;D Team Manager – Next Generation Grids Transformers 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>TD SYNNEX Switzerland GmbH</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Rotkreuz, Switzerland</t>
+          <t>Satigny, Geneva, Switzerland</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3738,15 +3766,15 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/83432ecd-3dd3-4a98-9663-6f678ad52a5e</t>
+          <t>https://www.jobup.ch/en/jobs/detail/5d31e1bb-71de-4d16-951e-a91f8a523888</t>
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>marketing, switzerland</t>
+          <t>geneva, marketing, switzerland</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -3756,7 +3784,7 @@
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3768,17 +3796,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Global Medical Director Cardiometabolic</t>
+          <t>Project Management Portfolio Manager 80 – 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Abbott AG</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Switzerland &amp;gt; Allschwil : H-127</t>
+          <t>Turgi, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -3788,11 +3816,11 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9e624f50-f1d8-4017-b805-17a8f78d7acd</t>
+          <t>https://www.jobup.ch/en/jobs/detail/8346982e-831d-451c-980b-0c74cdfa2987</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -3801,12 +3829,12 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>director</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3818,35 +3846,31 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Finance and Administration Manager</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Fairmont Grand Hôtel Geneva</t>
-        </is>
-      </c>
+          <t>Digital Marketing Manager - English</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Hotel Rotary Geneva - MGallery, Geneva, Switzerland</t>
+          <t>Limburg</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/0996602f-337e-48a0-a447-50bc3dbec7b2</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/marketing-pr-positions/digital-marketing-manager-english/wp7kjAdTkg5FeoRExbUjSA</t>
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>geneva, marketing, switzerland</t>
+          <t>marketing, netherlands</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -3856,7 +3880,7 @@
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3868,35 +3892,35 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>R&amp;D Team Manager – Next Generation Grids Transformers 80 - 100% (f/m/d)</t>
+          <t>Performance Marketing Manager</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>Lecram Marketing GmbH</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Satigny, Geneva, Switzerland</t>
+          <t>Müllheim</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/5d31e1bb-71de-4d16-951e-a91f8a523888</t>
+          <t>https://www.arbeitnow.com/jobs/companies/lecram-marketing-gmbh/performance-marketing-manager-mullheim-46821</t>
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>geneva, marketing, switzerland</t>
+          <t>germany, marketing</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -3906,7 +3930,7 @@
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3918,45 +3942,45 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Project Management Portfolio Manager 80 – 100% (f/m/d)</t>
+          <t>Marketing Lead (m/w/d)</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>ocumeda GmbH</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Turgi, Aargau, Switzerland</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/8346982e-831d-451c-980b-0c74cdfa2987</t>
+          <t>https://www.arbeitnow.com/jobs/companies/ocumeda-gmbh/marketing-lead-munich-132881</t>
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>marketing, switzerland</t>
+          <t>germany, marketing, munich</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>lead</t>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -3968,17 +3992,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Performance Marketing Manager</t>
+          <t>Performance Marketing Manager - Google Ads</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Lecram Marketing GmbH</t>
+          <t>Every.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Müllheim</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -3988,15 +4012,15 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/lecram-marketing-gmbh/performance-marketing-manager-mullheim-46821</t>
+          <t>https://www.arbeitnow.com/jobs/companies/every/performance-marketing-manager-google-ads-berlin-391005</t>
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>berlin, germany, marketing</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4006,7 +4030,7 @@
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4018,17 +4042,17 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Marketing Lead (m/w/d)</t>
+          <t>Online Marketing Projektmanager (m/w/d)</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>ocumeda GmbH</t>
+          <t>Shopwise GmbH</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -4038,25 +4062,25 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/ocumeda-gmbh/marketing-lead-munich-132881</t>
+          <t>https://www.arbeitnow.com/jobs/companies/shopwise-gmbh/online-marketing-projektmanager-berlin-351214</t>
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich</t>
+          <t>berlin, germany, marketing</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>lead</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4068,12 +4092,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Performance Marketing Manager - Google Ads</t>
+          <t>Director of Brand Marketing (m/f/d)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Every.</t>
+          <t>raisin</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -4088,11 +4112,11 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/every/performance-marketing-manager-google-ads-berlin-391005</t>
+          <t>https://www.arbeitnow.com/jobs/companies/raisin/director-of-brand-marketing-berlin-73818</t>
         </is>
       </c>
       <c r="G79" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -4101,12 +4125,12 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>director</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4118,17 +4142,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Online Marketing Projektmanager (m/w/d)</t>
+          <t>Influencer Marketing Manager (m/w/d) - YouTube</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Shopwise GmbH</t>
+          <t>Adspace</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -4138,15 +4162,15 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/shopwise-gmbh/online-marketing-projektmanager-berlin-351214</t>
+          <t>https://www.arbeitnow.com/jobs/companies/adspace/influencer-marketing-manager-youtube-hamburg-255974</t>
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>germany, hamburg, marketing</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -4156,7 +4180,7 @@
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4168,17 +4192,17 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Director of Brand Marketing (m/f/d)</t>
+          <t>Marketing Manager (w/m/d) Brand &amp; Content</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>raisin</t>
+          <t>Skalar</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -4188,25 +4212,25 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/raisin/director-of-brand-marketing-berlin-73818</t>
+          <t>https://www.arbeitnow.com/jobs/companies/skalar/marketing-manager-brand-content-munich-92852</t>
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>germany, marketing, munich</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>director</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4218,17 +4242,17 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Influencer Marketing Manager (m/w/d) - YouTube</t>
+          <t>Performance Marketing Manager (m/w/d)</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Adspace</t>
+          <t>Just Hiring</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -4238,15 +4262,15 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/adspace/influencer-marketing-manager-youtube-hamburg-255974</t>
+          <t>https://www.arbeitnow.com/jobs/companies/just-hiring/paid-media-manager-berlin-461575</t>
         </is>
       </c>
       <c r="G82" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>germany, hamburg, marketing</t>
+          <t>berlin, germany, marketing</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4256,7 +4280,7 @@
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4268,45 +4292,41 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Teamlead CRM (Marketing) (m/w/d)</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>PERRCON job network</t>
-        </is>
-      </c>
+          <t>Assistant Financial Controller | English | Almere area</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Bremen</t>
+          <t>Almere</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/perrcon-job-network/teamlead-crm-marketing-bremen-422984</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/finance-accounting-positions/assistant-financial-controller-english-almere-area/io2zwMAJH8NAJsCQGtpojm</t>
         </is>
       </c>
       <c r="G83" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>netherlands</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>lead</t>
+          <t>accounting</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4318,45 +4338,41 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Marketing Manager (w/m/d) Brand &amp; Content</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Skalar</t>
-        </is>
-      </c>
+          <t>Senior Export Desk Representative | English | Nijmegen</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Nijmegen</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/skalar/marketing-manager-brand-content-munich-92852</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/supply-chain-logistics-positions/senior-export-desk-representative-english-nijmegen/eZHBB8zzfMrpU33E1wJL7y</t>
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich</t>
+          <t>netherlands</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>senior</t>
         </is>
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4368,45 +4384,41 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Performance Marketing Manager (m/w/d)</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Just Hiring</t>
-        </is>
-      </c>
+          <t>Java Backend Engineer (Kotlin) - Freelance/zzp</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/just-hiring/paid-media-manager-berlin-461575</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/java-backend-engineer-kotlin-freelancezzp/kP1rMZUuK5tXV3FkBKWGuV</t>
         </is>
       </c>
       <c r="G85" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>amsterdam, netherlands</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>backend engineer</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4418,13 +4430,13 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Digital Marketing Manager - English</t>
+          <t>Java Backend Engineer (Kotlin) - Temporary</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Limburg</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -4434,25 +4446,25 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/marketing-pr-positions/digital-marketing-manager-english/wp7kjAdTkg5FeoRExbUjSA</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/java-backend-engineer-kotlin-temporary/oQs6kAvwDoSinBavtghURc</t>
         </is>
       </c>
       <c r="G86" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>marketing, netherlands</t>
+          <t>amsterdam, netherlands</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>backend engineer</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4464,27 +4476,23 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Manager (m/w/d)</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>ocumeda GmbH</t>
-        </is>
-      </c>
+          <t>DevOps Engineer - SIP Core (Voice Platform)</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>Rotterdam Temporary</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Arbeitnow Marketing Germany</t>
+          <t>IamExpat Jobs Netherlands</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/ocumeda-gmbh/senior-marketing-manager-munich-300276</t>
+          <t>https://www.iamexpat.nl/career/jobs-netherlands/it-technology-positions/devops-engineer-sip-core-voice-platform/sGfXBGvCBQ2Vdqa6CTH62X</t>
         </is>
       </c>
       <c r="G87" s="2" t="n">
@@ -4492,17 +4500,17 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich</t>
+          <t>netherlands, rotterdam</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>manager, senior</t>
+          <t>devops</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4514,17 +4522,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Senior Performance Marketing Manager 100% remote (m/w/d)</t>
+          <t>Senior Marketing Manager (m/w/d)</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>KX Marketing</t>
+          <t>ocumeda GmbH</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Würselen</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4534,7 +4542,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/kx-marketing/projektleiter-kundenbetreuer-im-performance-marketing-100-remote-wurselen-159573</t>
+          <t>https://www.arbeitnow.com/jobs/companies/ocumeda-gmbh/senior-marketing-manager-munich-300276</t>
         </is>
       </c>
       <c r="G88" s="2" t="n">
@@ -4542,7 +4550,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, remote</t>
+          <t>germany, marketing, munich</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -4552,7 +4560,7 @@
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4564,17 +4572,17 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Senior Marketing Manager (m/w/d)</t>
+          <t>Senior Performance Marketing Manager 100% remote (m/w/d)</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>CKM Group</t>
+          <t>KX Marketing</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Würselen</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -4584,7 +4592,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/ckm-group/marketing-manager-berlin-250367</t>
+          <t>https://www.arbeitnow.com/jobs/companies/kx-marketing/projektleiter-kundenbetreuer-im-performance-marketing-100-remote-wurselen-159573</t>
         </is>
       </c>
       <c r="G89" s="2" t="n">
@@ -4592,7 +4600,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, marketing</t>
+          <t>germany, marketing, remote</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -4602,7 +4610,7 @@
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4614,12 +4622,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>B2B Marketing Manager (m/w/x)</t>
+          <t>Senior Marketing Manager (m/w/d)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Bring! Labs AG</t>
+          <t>CKM Group</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4634,7 +4642,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bring-labs-ag/senior-b2b-content-growth-marketing-manager-befristet-bis-jan-2028-alle-berlin-27533</t>
+          <t>https://www.arbeitnow.com/jobs/companies/ckm-group/marketing-manager-berlin-250367</t>
         </is>
       </c>
       <c r="G90" s="2" t="n">
@@ -4642,7 +4650,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, growth, marketing</t>
+          <t>berlin, germany, marketing</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -4652,7 +4660,7 @@
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4664,17 +4672,17 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Senior Performance Marketing Manager (m/w/d)</t>
+          <t>B2B Marketing Manager (m/w/x)</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>FINE DINE Verlags GmbH</t>
+          <t>Bring! Labs AG</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Ulm</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -4684,7 +4692,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fine-dine-verlags-gmbh/senior-performance-marketing-manager-ulm-271620</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bring-labs-ag/senior-b2b-content-growth-marketing-manager-befristet-bis-jan-2028-alle-berlin-27533</t>
         </is>
       </c>
       <c r="G91" s="2" t="n">
@@ -4692,7 +4700,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing</t>
+          <t>berlin, germany, growth, marketing</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -4702,7 +4710,7 @@
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; seniority warning</t>
+          <t>target location; seniority warning</t>
         </is>
       </c>
     </row>
@@ -4714,23 +4722,27 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Senior Export Desk Representative | English | Nijmegen</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr"/>
+          <t>Senior Performance Marketing Manager (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>FINE DINE Verlags GmbH</t>
+        </is>
+      </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Nijmegen</t>
+          <t>Ulm</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>IamExpat Jobs Netherlands</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.nl/career/jobs-netherlands/supply-chain-logistics-positions/senior-export-desk-representative-english-nijmegen/eZHBB8zzfMrpU33E1wJL7y</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fine-dine-verlags-gmbh/senior-performance-marketing-manager-ulm-271620</t>
         </is>
       </c>
       <c r="G92" s="2" t="n">
@@ -4738,12 +4750,12 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>netherlands</t>
+          <t>germany, marketing</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>senior</t>
+          <t>manager, senior</t>
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add daily GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/daily_jobs.xlsx
+++ b/daily_jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Daily Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Jobs'!$A$1:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Jobs'!$A$1:$J$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -513,22 +513,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Internship - DAT Industrialization</t>
+          <t>Internship Application Development 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>SR Technics Switzerland AG</t>
+          <t>Hitachi Energy AG</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Switzerland, Zürich</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/c6014db5-c37c-4b5f-b37c-2333b1f58759</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/61d3dd89-eaff-4dcc-b9b7-2b08c0d7e8c2</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>business development, intern, internship, switzerland</t>
+          <t>business development, intern, internship, switzerland, zurich</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -559,20 +559,24 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Working Student (x|f|m)</t>
+          <t>Internship in Low-Code Development 80 - 100% (f/m(d)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Sartorius Stedim Switzerland AG</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
+          <t>Hitachi Energy AG</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Dietlikon, Zurich, Switzerland</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>jobs.ch Business Development Switzerland</t>
@@ -580,15 +584,15 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobs.ch/en/vacancies/detail/0c1cfb78-2bf7-4029-a0cc-b8a91ea7830f</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/bf373b79-6d8c-4c0b-beef-d480605b70fe</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>business development, switzerland, working student</t>
+          <t>business development, intern, internship, switzerland, zurich</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -601,58 +605,54 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Internship in Digital Media Tracking 80 - 100% (f/m/d)</t>
+          <t>Working Student (x|f|m)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Zurich, Zurich, Switzerland</t>
-        </is>
-      </c>
+          <t>Sartorius Stedim Switzerland AG</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>jobs.ch Business Development Switzerland</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/fef9024a-a85f-451f-bdad-bece70b5715c</t>
+          <t>https://www.jobs.ch/en/vacancies/detail/0c1cfb78-2bf7-4029-a0cc-b8a91ea7830f</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>intern, internship, marketing, switzerland, zurich</t>
+          <t>business development, switzerland, working student</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit</t>
+          <t>role fit; strong keyword match; target location; junior/internship fit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Internship in IT Onsite Support 80 - 100% (f/m/d)</t>
+          <t>Internship in Digital Media Tracking 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Baden, Aargau, Switzerland</t>
+          <t>Zurich, Zurich, Switzerland</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9a77c54c-fdf6-4004-b6d5-b57462d218c5</t>
+          <t>https://www.jobup.ch/en/jobs/detail/fef9024a-a85f-451f-bdad-bece70b5715c</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
@@ -680,7 +680,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>intern, internship, marketing, switzerland</t>
+          <t>intern, internship, marketing, switzerland, zurich</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -693,12 +693,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Internship Application Development 80 - 100% (f/m/d)</t>
+          <t>Internship in IT Onsite Support 80 - 100% (f/m/d)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Zurich, Zurich, Switzerland</t>
+          <t>Baden, Aargau, Switzerland</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/61d3dd89-eaff-4dcc-b9b7-2b08c0d7e8c2</t>
+          <t>https://www.jobup.ch/en/jobs/detail/9a77c54c-fdf6-4004-b6d5-b57462d218c5</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>intern, internship, marketing, switzerland, zurich</t>
+          <t>intern, internship, marketing, switzerland</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -739,68 +739,68 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Internship in Low-Code Development 80 - 100% (f/m(d)</t>
+          <t>Working Student Marketing (m/f/x)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Energy AG</t>
+          <t>CRX Markets AG</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Dietlikon, Zurich, Switzerland</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/bf373b79-6d8c-4c0b-beef-d480605b70fe</t>
+          <t>https://www.arbeitnow.com/jobs/companies/crx-markets-ag/working-student-marketing-munich-132586</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>intern, internship, marketing, switzerland, zurich</t>
+          <t>germany, marketing, munich, working student</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit</t>
+          <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Fielde Marketing &amp; Community Outreach internship</t>
+          <t>Online Marketing Trainee</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Punto Cubano Berlin</t>
+          <t>Cyrus Digital GmbH</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -810,118 +810,26 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/punto-cubano-berlin/fielde-marketing-community-outreach-internship-berlin-329034</t>
+          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>berlin, germany, intern, internship, marketing</t>
+          <t>germany, marketing, munich, trainee</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>strong keyword match; target location; junior/internship fit</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Swibeco AG</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Lausanne, Waadt, Switzerland</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>jobup.ch Marketing Switzerland</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9d3f6b3d-8e94-4e58-9c54-694f9db91205</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>lausanne, marketing, switzerland, trainee</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>target location; junior/internship fit</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Online Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Cyrus Digital GmbH</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Arbeitnow Marketing Germany</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>germany, marketing, munich, trainee</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
           <t>target location; junior/internship fit</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
+  <autoFilter ref="A1:J8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -930,8 +838,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve IMAP mailbox selection
</commit_message>
<xml_diff>
--- a/daily_jobs.xlsx
+++ b/daily_jobs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Daily Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Jobs'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Jobs'!$A$1:$J$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -744,27 +744,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Marketing Trainee</t>
+          <t>Working Student Marketing (m/f/x)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Swibeco AG</t>
+          <t>CRX Markets AG</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Lausanne, Waadt, Switzerland</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>jobup.ch Marketing Switzerland</t>
+          <t>Arbeitnow Marketing Germany</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.jobup.ch/en/jobs/detail/9d3f6b3d-8e94-4e58-9c54-694f9db91205</t>
+          <t>https://www.arbeitnow.com/jobs/companies/crx-markets-ag/working-student-marketing-munich-132586</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>lausanne, marketing, switzerland, trainee</t>
+          <t>germany, marketing, munich, working student</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -790,12 +790,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Working Student Marketing (m/f/x)</t>
+          <t>Online Marketing Trainee</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CRX Markets AG</t>
+          <t>Cyrus Digital GmbH</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/crx-markets-ag/working-student-marketing-munich-132586</t>
+          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -818,7 +818,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>germany, marketing, munich, working student</t>
+          <t>germany, marketing, munich, trainee</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -828,54 +828,8 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Online Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Cyrus Digital GmbH</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Arbeitnow Marketing Germany</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.arbeitnow.com/jobs/companies/cyrus-digital-gmbh/online-marketing-trainee-munich-499188</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>germany, marketing, munich, trainee</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>target location; junior/internship fit</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -884,7 +838,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>